<commit_message>
Write an index.html linking the HTML reports
When HTML is among the output formats, a run now also writes an index.html
beside the reports: a table of contents linking to each team's report and to the
cross-team overview, with each team's own-rule, covering-rule and finding
counts. Opening the run's directory -- served over HTTP, or dropped on a file
share -- lands on a page to click through rather than a bare file listing. It
goes in the run's directory, so a timestamped run gets its own; it is written
only when html is a configured format, and it links only the reports that were
actually written, so --sample stays consistent.

The committed example is regenerated to include it. Only the timestamps and the
day-relative wording in findings move -- the estate is generated from a fixed
seed, so its content is unchanged.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/example/reports/00_OVERVIEW_all-teams.xlsx
+++ b/example/reports/00_OVERVIEW_all-teams.xlsx
@@ -44,7 +44,7 @@
     <t>Report generated</t>
   </si>
   <si>
-    <t>2026-07-30 19:26</t>
+    <t>2026-08-04 22:41</t>
   </si>
   <si>
     <t>Rules analysed</t>
@@ -1070,7 +1070,7 @@
     <t>Past its stated expiry date</t>
   </si>
   <si>
-    <t>The description gives an expiry of 2026-06-13, 47 days ago, but the rule is still active.</t>
+    <t>The description gives an expiry of 2026-06-13, 52 days ago, but the rule is still active.</t>
   </si>
   <si>
     <t>Remove the rule, or extend it with a new change reference.</t>
@@ -1163,7 +1163,7 @@
     <t>Expires soon</t>
   </si>
   <si>
-    <t>The stated expiry is 2026-08-27, in 28 days.</t>
+    <t>The stated expiry is 2026-08-27, in 23 days.</t>
   </si>
   <si>
     <t>Confirm whether the access is still needed before it lapses.</t>

</xml_diff>